<commit_message>
Windmill Poker - Phase 5: Spieler-Liste, Profil mit Bar-Chart, Gallerie + Re-Seed v2
Re-Seed aus Auszahlungen-Sheet (12 STs, ST11 19.02.26 inkl. Frank-Tagessieg
100€). Verify-v2 prueft jede Zelle gegen DB - Σ + Teilnahmen matchen exakt.

UI:
- /spieler: Spieler-Liste alphabetisch
- /spieler/[id]: Profil mit Stat-Karten, Platz-Badges, Bar-Chart mit Tagessieg-
  Hervorhebung, Spieltage-Tabelle (mockup-Vorgabe profil.html)
- /gallerie: Foto-Grid (Empty-State wenn keine Fotos), Kamera-Button
- /gallerie/[id]: Foto-Detail mit Kommentar + Bearbeiten-Button
- Sandige 4px-Scrollbar als .scroll-warm Utility (Tailwind 4 erfordert @layer)
- Spieltage-Liste mit ST11 als offen, scroll-warm

CLAUDE.md erweitert um Excel-Source-of-Truth (Auszahlungen-Sheet) und
0-Cell-Mehrdeutigkeit-Regel.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Windmill_Poker_results_test.xlsx
+++ b/Windmill_Poker_results_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\sandbox\Superpowers-Trial_one\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D60B6B1E-E3C7-4930-9F83-DA566A316593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085860E5-ABD4-4926-98B0-2DC0BE0C2799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2190,7 +2190,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="1177" row="2">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -2203,7 +2203,7 @@
     <we:reference id="wa200009404" version="1.0.0.5" store="wa200009404" storeType="OMEX"/>
   </we:alternateReferences>
   <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+    <we:property name="claude.fileId" value="&quot;3a6ccdda-b6bd-4566-8d5d-7072d59e33cc&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -14384,6 +14384,193 @@
     </row>
   </sheetData>
   <mergeCells count="198">
+    <mergeCell ref="W65:X65"/>
+    <mergeCell ref="Y65:Z65"/>
+    <mergeCell ref="AA65:AB65"/>
+    <mergeCell ref="AC65:AD65"/>
+    <mergeCell ref="I65:J65"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="O65:P65"/>
+    <mergeCell ref="Q65:R65"/>
+    <mergeCell ref="S65:T65"/>
+    <mergeCell ref="U65:V65"/>
+    <mergeCell ref="W66:X66"/>
+    <mergeCell ref="Y66:Z66"/>
+    <mergeCell ref="AA66:AB66"/>
+    <mergeCell ref="AC66:AD66"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="K66:L66"/>
+    <mergeCell ref="M66:N66"/>
+    <mergeCell ref="O66:P66"/>
+    <mergeCell ref="Q66:R66"/>
+    <mergeCell ref="S66:T66"/>
+    <mergeCell ref="U66:V66"/>
+    <mergeCell ref="W75:X75"/>
+    <mergeCell ref="Y75:Z75"/>
+    <mergeCell ref="AA75:AB75"/>
+    <mergeCell ref="AC75:AD75"/>
+    <mergeCell ref="I75:J75"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="M75:N75"/>
+    <mergeCell ref="O75:P75"/>
+    <mergeCell ref="Q75:R75"/>
+    <mergeCell ref="S75:T75"/>
+    <mergeCell ref="U75:V75"/>
+    <mergeCell ref="W76:X76"/>
+    <mergeCell ref="Y76:Z76"/>
+    <mergeCell ref="AA76:AB76"/>
+    <mergeCell ref="AC76:AD76"/>
+    <mergeCell ref="I76:J76"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="M76:N76"/>
+    <mergeCell ref="O76:P76"/>
+    <mergeCell ref="Q76:R76"/>
+    <mergeCell ref="S76:T76"/>
+    <mergeCell ref="U76:V76"/>
+    <mergeCell ref="W85:X85"/>
+    <mergeCell ref="Y85:Z85"/>
+    <mergeCell ref="AA85:AB85"/>
+    <mergeCell ref="AC85:AD85"/>
+    <mergeCell ref="I85:J85"/>
+    <mergeCell ref="K85:L85"/>
+    <mergeCell ref="M85:N85"/>
+    <mergeCell ref="O85:P85"/>
+    <mergeCell ref="Q85:R85"/>
+    <mergeCell ref="S85:T85"/>
+    <mergeCell ref="U85:V85"/>
+    <mergeCell ref="W86:X86"/>
+    <mergeCell ref="Y86:Z86"/>
+    <mergeCell ref="AA86:AB86"/>
+    <mergeCell ref="AC86:AD86"/>
+    <mergeCell ref="I86:J86"/>
+    <mergeCell ref="K86:L86"/>
+    <mergeCell ref="M86:N86"/>
+    <mergeCell ref="O86:P86"/>
+    <mergeCell ref="Q86:R86"/>
+    <mergeCell ref="S86:T86"/>
+    <mergeCell ref="U86:V86"/>
+    <mergeCell ref="W95:X95"/>
+    <mergeCell ref="Y95:Z95"/>
+    <mergeCell ref="AA95:AB95"/>
+    <mergeCell ref="AC95:AD95"/>
+    <mergeCell ref="I95:J95"/>
+    <mergeCell ref="K95:L95"/>
+    <mergeCell ref="M95:N95"/>
+    <mergeCell ref="O95:P95"/>
+    <mergeCell ref="Q95:R95"/>
+    <mergeCell ref="S95:T95"/>
+    <mergeCell ref="U95:V95"/>
+    <mergeCell ref="W13:X13"/>
+    <mergeCell ref="Y13:Z13"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AC13:AD13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="W14:X14"/>
+    <mergeCell ref="Y14:Z14"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="AC14:AD14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="S14:T14"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="W23:X23"/>
+    <mergeCell ref="Y23:Z23"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AC23:AD23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="S23:T23"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="W96:X96"/>
+    <mergeCell ref="Y96:Z96"/>
+    <mergeCell ref="AA96:AB96"/>
+    <mergeCell ref="AC96:AD96"/>
+    <mergeCell ref="I96:J96"/>
+    <mergeCell ref="K96:L96"/>
+    <mergeCell ref="M96:N96"/>
+    <mergeCell ref="O96:P96"/>
+    <mergeCell ref="Q96:R96"/>
+    <mergeCell ref="S96:T96"/>
+    <mergeCell ref="U96:V96"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="W33:X33"/>
+    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="AA33:AB33"/>
+    <mergeCell ref="AC33:AD33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:R33"/>
+    <mergeCell ref="S33:T33"/>
+    <mergeCell ref="U33:V33"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="AA34:AB34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="U34:V34"/>
+    <mergeCell ref="W43:X43"/>
+    <mergeCell ref="Y43:Z43"/>
+    <mergeCell ref="AA43:AB43"/>
+    <mergeCell ref="AC43:AD43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="M43:N43"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="Q43:R43"/>
+    <mergeCell ref="S43:T43"/>
+    <mergeCell ref="U43:V43"/>
+    <mergeCell ref="W44:X44"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="AA44:AB44"/>
+    <mergeCell ref="AC44:AD44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="U44:V44"/>
+    <mergeCell ref="W53:X53"/>
+    <mergeCell ref="Y53:Z53"/>
+    <mergeCell ref="AA53:AB53"/>
+    <mergeCell ref="AC53:AD53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="K53:L53"/>
+    <mergeCell ref="M53:N53"/>
+    <mergeCell ref="O53:P53"/>
+    <mergeCell ref="Q53:R53"/>
+    <mergeCell ref="S53:T53"/>
+    <mergeCell ref="U53:V53"/>
     <mergeCell ref="W54:X54"/>
     <mergeCell ref="Y54:Z54"/>
     <mergeCell ref="AA54:AB54"/>
@@ -14395,193 +14582,6 @@
     <mergeCell ref="Q54:R54"/>
     <mergeCell ref="S54:T54"/>
     <mergeCell ref="U54:V54"/>
-    <mergeCell ref="W53:X53"/>
-    <mergeCell ref="Y53:Z53"/>
-    <mergeCell ref="AA53:AB53"/>
-    <mergeCell ref="AC53:AD53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="K53:L53"/>
-    <mergeCell ref="M53:N53"/>
-    <mergeCell ref="O53:P53"/>
-    <mergeCell ref="Q53:R53"/>
-    <mergeCell ref="S53:T53"/>
-    <mergeCell ref="U53:V53"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="AA44:AB44"/>
-    <mergeCell ref="AC44:AD44"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="O44:P44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="U44:V44"/>
-    <mergeCell ref="W43:X43"/>
-    <mergeCell ref="Y43:Z43"/>
-    <mergeCell ref="AA43:AB43"/>
-    <mergeCell ref="AC43:AD43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="M43:N43"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="Q43:R43"/>
-    <mergeCell ref="S43:T43"/>
-    <mergeCell ref="U43:V43"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="AA34:AB34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="U34:V34"/>
-    <mergeCell ref="W33:X33"/>
-    <mergeCell ref="Y33:Z33"/>
-    <mergeCell ref="AA33:AB33"/>
-    <mergeCell ref="AC33:AD33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:R33"/>
-    <mergeCell ref="S33:T33"/>
-    <mergeCell ref="U33:V33"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="W96:X96"/>
-    <mergeCell ref="Y96:Z96"/>
-    <mergeCell ref="AA96:AB96"/>
-    <mergeCell ref="AC96:AD96"/>
-    <mergeCell ref="I96:J96"/>
-    <mergeCell ref="K96:L96"/>
-    <mergeCell ref="M96:N96"/>
-    <mergeCell ref="O96:P96"/>
-    <mergeCell ref="Q96:R96"/>
-    <mergeCell ref="S96:T96"/>
-    <mergeCell ref="U96:V96"/>
-    <mergeCell ref="W23:X23"/>
-    <mergeCell ref="Y23:Z23"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AC23:AD23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="S23:T23"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="W14:X14"/>
-    <mergeCell ref="Y14:Z14"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="AC14:AD14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="S14:T14"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="W13:X13"/>
-    <mergeCell ref="Y13:Z13"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AC13:AD13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="S13:T13"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="W95:X95"/>
-    <mergeCell ref="Y95:Z95"/>
-    <mergeCell ref="AA95:AB95"/>
-    <mergeCell ref="AC95:AD95"/>
-    <mergeCell ref="I95:J95"/>
-    <mergeCell ref="K95:L95"/>
-    <mergeCell ref="M95:N95"/>
-    <mergeCell ref="O95:P95"/>
-    <mergeCell ref="Q95:R95"/>
-    <mergeCell ref="S95:T95"/>
-    <mergeCell ref="U95:V95"/>
-    <mergeCell ref="W86:X86"/>
-    <mergeCell ref="Y86:Z86"/>
-    <mergeCell ref="AA86:AB86"/>
-    <mergeCell ref="AC86:AD86"/>
-    <mergeCell ref="I86:J86"/>
-    <mergeCell ref="K86:L86"/>
-    <mergeCell ref="M86:N86"/>
-    <mergeCell ref="O86:P86"/>
-    <mergeCell ref="Q86:R86"/>
-    <mergeCell ref="S86:T86"/>
-    <mergeCell ref="U86:V86"/>
-    <mergeCell ref="W85:X85"/>
-    <mergeCell ref="Y85:Z85"/>
-    <mergeCell ref="AA85:AB85"/>
-    <mergeCell ref="AC85:AD85"/>
-    <mergeCell ref="I85:J85"/>
-    <mergeCell ref="K85:L85"/>
-    <mergeCell ref="M85:N85"/>
-    <mergeCell ref="O85:P85"/>
-    <mergeCell ref="Q85:R85"/>
-    <mergeCell ref="S85:T85"/>
-    <mergeCell ref="U85:V85"/>
-    <mergeCell ref="W76:X76"/>
-    <mergeCell ref="Y76:Z76"/>
-    <mergeCell ref="AA76:AB76"/>
-    <mergeCell ref="AC76:AD76"/>
-    <mergeCell ref="I76:J76"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="M76:N76"/>
-    <mergeCell ref="O76:P76"/>
-    <mergeCell ref="Q76:R76"/>
-    <mergeCell ref="S76:T76"/>
-    <mergeCell ref="U76:V76"/>
-    <mergeCell ref="W75:X75"/>
-    <mergeCell ref="Y75:Z75"/>
-    <mergeCell ref="AA75:AB75"/>
-    <mergeCell ref="AC75:AD75"/>
-    <mergeCell ref="I75:J75"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="M75:N75"/>
-    <mergeCell ref="O75:P75"/>
-    <mergeCell ref="Q75:R75"/>
-    <mergeCell ref="S75:T75"/>
-    <mergeCell ref="U75:V75"/>
-    <mergeCell ref="W66:X66"/>
-    <mergeCell ref="Y66:Z66"/>
-    <mergeCell ref="AA66:AB66"/>
-    <mergeCell ref="AC66:AD66"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="K66:L66"/>
-    <mergeCell ref="M66:N66"/>
-    <mergeCell ref="O66:P66"/>
-    <mergeCell ref="Q66:R66"/>
-    <mergeCell ref="S66:T66"/>
-    <mergeCell ref="U66:V66"/>
-    <mergeCell ref="W65:X65"/>
-    <mergeCell ref="Y65:Z65"/>
-    <mergeCell ref="AA65:AB65"/>
-    <mergeCell ref="AC65:AD65"/>
-    <mergeCell ref="I65:J65"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="O65:P65"/>
-    <mergeCell ref="Q65:R65"/>
-    <mergeCell ref="S65:T65"/>
-    <mergeCell ref="U65:V65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -20731,6 +20731,193 @@
     <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="198">
+    <mergeCell ref="W65:X65"/>
+    <mergeCell ref="Y65:Z65"/>
+    <mergeCell ref="AA65:AB65"/>
+    <mergeCell ref="AC65:AD65"/>
+    <mergeCell ref="I65:J65"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="M65:N65"/>
+    <mergeCell ref="O65:P65"/>
+    <mergeCell ref="Q65:R65"/>
+    <mergeCell ref="S65:T65"/>
+    <mergeCell ref="U65:V65"/>
+    <mergeCell ref="W66:X66"/>
+    <mergeCell ref="Y66:Z66"/>
+    <mergeCell ref="AA66:AB66"/>
+    <mergeCell ref="AC66:AD66"/>
+    <mergeCell ref="I66:J66"/>
+    <mergeCell ref="K66:L66"/>
+    <mergeCell ref="M66:N66"/>
+    <mergeCell ref="O66:P66"/>
+    <mergeCell ref="Q66:R66"/>
+    <mergeCell ref="S66:T66"/>
+    <mergeCell ref="U66:V66"/>
+    <mergeCell ref="W75:X75"/>
+    <mergeCell ref="Y75:Z75"/>
+    <mergeCell ref="AA75:AB75"/>
+    <mergeCell ref="AC75:AD75"/>
+    <mergeCell ref="I75:J75"/>
+    <mergeCell ref="K75:L75"/>
+    <mergeCell ref="M75:N75"/>
+    <mergeCell ref="O75:P75"/>
+    <mergeCell ref="Q75:R75"/>
+    <mergeCell ref="S75:T75"/>
+    <mergeCell ref="U75:V75"/>
+    <mergeCell ref="W76:X76"/>
+    <mergeCell ref="Y76:Z76"/>
+    <mergeCell ref="AA76:AB76"/>
+    <mergeCell ref="AC76:AD76"/>
+    <mergeCell ref="I76:J76"/>
+    <mergeCell ref="K76:L76"/>
+    <mergeCell ref="M76:N76"/>
+    <mergeCell ref="O76:P76"/>
+    <mergeCell ref="Q76:R76"/>
+    <mergeCell ref="S76:T76"/>
+    <mergeCell ref="U76:V76"/>
+    <mergeCell ref="W85:X85"/>
+    <mergeCell ref="Y85:Z85"/>
+    <mergeCell ref="AA85:AB85"/>
+    <mergeCell ref="AC85:AD85"/>
+    <mergeCell ref="I85:J85"/>
+    <mergeCell ref="K85:L85"/>
+    <mergeCell ref="M85:N85"/>
+    <mergeCell ref="O85:P85"/>
+    <mergeCell ref="Q85:R85"/>
+    <mergeCell ref="S85:T85"/>
+    <mergeCell ref="U85:V85"/>
+    <mergeCell ref="W86:X86"/>
+    <mergeCell ref="Y86:Z86"/>
+    <mergeCell ref="AA86:AB86"/>
+    <mergeCell ref="AC86:AD86"/>
+    <mergeCell ref="I86:J86"/>
+    <mergeCell ref="K86:L86"/>
+    <mergeCell ref="M86:N86"/>
+    <mergeCell ref="O86:P86"/>
+    <mergeCell ref="Q86:R86"/>
+    <mergeCell ref="S86:T86"/>
+    <mergeCell ref="U86:V86"/>
+    <mergeCell ref="W95:X95"/>
+    <mergeCell ref="Y95:Z95"/>
+    <mergeCell ref="AA95:AB95"/>
+    <mergeCell ref="AC95:AD95"/>
+    <mergeCell ref="I95:J95"/>
+    <mergeCell ref="K95:L95"/>
+    <mergeCell ref="M95:N95"/>
+    <mergeCell ref="O95:P95"/>
+    <mergeCell ref="Q95:R95"/>
+    <mergeCell ref="S95:T95"/>
+    <mergeCell ref="U95:V95"/>
+    <mergeCell ref="W13:X13"/>
+    <mergeCell ref="Y13:Z13"/>
+    <mergeCell ref="AA13:AB13"/>
+    <mergeCell ref="AC13:AD13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="W14:X14"/>
+    <mergeCell ref="Y14:Z14"/>
+    <mergeCell ref="AA14:AB14"/>
+    <mergeCell ref="AC14:AD14"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="S14:T14"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="W23:X23"/>
+    <mergeCell ref="Y23:Z23"/>
+    <mergeCell ref="AA23:AB23"/>
+    <mergeCell ref="AC23:AD23"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="S23:T23"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="W96:X96"/>
+    <mergeCell ref="Y96:Z96"/>
+    <mergeCell ref="AA96:AB96"/>
+    <mergeCell ref="AC96:AD96"/>
+    <mergeCell ref="I96:J96"/>
+    <mergeCell ref="K96:L96"/>
+    <mergeCell ref="M96:N96"/>
+    <mergeCell ref="O96:P96"/>
+    <mergeCell ref="Q96:R96"/>
+    <mergeCell ref="S96:T96"/>
+    <mergeCell ref="U96:V96"/>
+    <mergeCell ref="W24:X24"/>
+    <mergeCell ref="Y24:Z24"/>
+    <mergeCell ref="AA24:AB24"/>
+    <mergeCell ref="AC24:AD24"/>
+    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="M24:N24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="W33:X33"/>
+    <mergeCell ref="Y33:Z33"/>
+    <mergeCell ref="AA33:AB33"/>
+    <mergeCell ref="AC33:AD33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="Q33:R33"/>
+    <mergeCell ref="S33:T33"/>
+    <mergeCell ref="U33:V33"/>
+    <mergeCell ref="W34:X34"/>
+    <mergeCell ref="Y34:Z34"/>
+    <mergeCell ref="AA34:AB34"/>
+    <mergeCell ref="AC34:AD34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="M34:N34"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="U34:V34"/>
+    <mergeCell ref="W43:X43"/>
+    <mergeCell ref="Y43:Z43"/>
+    <mergeCell ref="AA43:AB43"/>
+    <mergeCell ref="AC43:AD43"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="K43:L43"/>
+    <mergeCell ref="M43:N43"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="Q43:R43"/>
+    <mergeCell ref="S43:T43"/>
+    <mergeCell ref="U43:V43"/>
+    <mergeCell ref="W44:X44"/>
+    <mergeCell ref="Y44:Z44"/>
+    <mergeCell ref="AA44:AB44"/>
+    <mergeCell ref="AC44:AD44"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="K44:L44"/>
+    <mergeCell ref="M44:N44"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="S44:T44"/>
+    <mergeCell ref="U44:V44"/>
+    <mergeCell ref="W53:X53"/>
+    <mergeCell ref="Y53:Z53"/>
+    <mergeCell ref="AA53:AB53"/>
+    <mergeCell ref="AC53:AD53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="K53:L53"/>
+    <mergeCell ref="M53:N53"/>
+    <mergeCell ref="O53:P53"/>
+    <mergeCell ref="Q53:R53"/>
+    <mergeCell ref="S53:T53"/>
+    <mergeCell ref="U53:V53"/>
     <mergeCell ref="W54:X54"/>
     <mergeCell ref="Y54:Z54"/>
     <mergeCell ref="AA54:AB54"/>
@@ -20742,193 +20929,6 @@
     <mergeCell ref="Q54:R54"/>
     <mergeCell ref="S54:T54"/>
     <mergeCell ref="U54:V54"/>
-    <mergeCell ref="W53:X53"/>
-    <mergeCell ref="Y53:Z53"/>
-    <mergeCell ref="AA53:AB53"/>
-    <mergeCell ref="AC53:AD53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="K53:L53"/>
-    <mergeCell ref="M53:N53"/>
-    <mergeCell ref="O53:P53"/>
-    <mergeCell ref="Q53:R53"/>
-    <mergeCell ref="S53:T53"/>
-    <mergeCell ref="U53:V53"/>
-    <mergeCell ref="W44:X44"/>
-    <mergeCell ref="Y44:Z44"/>
-    <mergeCell ref="AA44:AB44"/>
-    <mergeCell ref="AC44:AD44"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="K44:L44"/>
-    <mergeCell ref="M44:N44"/>
-    <mergeCell ref="O44:P44"/>
-    <mergeCell ref="Q44:R44"/>
-    <mergeCell ref="S44:T44"/>
-    <mergeCell ref="U44:V44"/>
-    <mergeCell ref="W43:X43"/>
-    <mergeCell ref="Y43:Z43"/>
-    <mergeCell ref="AA43:AB43"/>
-    <mergeCell ref="AC43:AD43"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="K43:L43"/>
-    <mergeCell ref="M43:N43"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="Q43:R43"/>
-    <mergeCell ref="S43:T43"/>
-    <mergeCell ref="U43:V43"/>
-    <mergeCell ref="W34:X34"/>
-    <mergeCell ref="Y34:Z34"/>
-    <mergeCell ref="AA34:AB34"/>
-    <mergeCell ref="AC34:AD34"/>
-    <mergeCell ref="I34:J34"/>
-    <mergeCell ref="K34:L34"/>
-    <mergeCell ref="M34:N34"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="Q34:R34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="U34:V34"/>
-    <mergeCell ref="W33:X33"/>
-    <mergeCell ref="Y33:Z33"/>
-    <mergeCell ref="AA33:AB33"/>
-    <mergeCell ref="AC33:AD33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="Q33:R33"/>
-    <mergeCell ref="S33:T33"/>
-    <mergeCell ref="U33:V33"/>
-    <mergeCell ref="W24:X24"/>
-    <mergeCell ref="Y24:Z24"/>
-    <mergeCell ref="AA24:AB24"/>
-    <mergeCell ref="AC24:AD24"/>
-    <mergeCell ref="I24:J24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="M24:N24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="W96:X96"/>
-    <mergeCell ref="Y96:Z96"/>
-    <mergeCell ref="AA96:AB96"/>
-    <mergeCell ref="AC96:AD96"/>
-    <mergeCell ref="I96:J96"/>
-    <mergeCell ref="K96:L96"/>
-    <mergeCell ref="M96:N96"/>
-    <mergeCell ref="O96:P96"/>
-    <mergeCell ref="Q96:R96"/>
-    <mergeCell ref="S96:T96"/>
-    <mergeCell ref="U96:V96"/>
-    <mergeCell ref="W23:X23"/>
-    <mergeCell ref="Y23:Z23"/>
-    <mergeCell ref="AA23:AB23"/>
-    <mergeCell ref="AC23:AD23"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="M23:N23"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="S23:T23"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="W14:X14"/>
-    <mergeCell ref="Y14:Z14"/>
-    <mergeCell ref="AA14:AB14"/>
-    <mergeCell ref="AC14:AD14"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="S14:T14"/>
-    <mergeCell ref="U14:V14"/>
-    <mergeCell ref="W13:X13"/>
-    <mergeCell ref="Y13:Z13"/>
-    <mergeCell ref="AA13:AB13"/>
-    <mergeCell ref="AC13:AD13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="S13:T13"/>
-    <mergeCell ref="U13:V13"/>
-    <mergeCell ref="W95:X95"/>
-    <mergeCell ref="Y95:Z95"/>
-    <mergeCell ref="AA95:AB95"/>
-    <mergeCell ref="AC95:AD95"/>
-    <mergeCell ref="I95:J95"/>
-    <mergeCell ref="K95:L95"/>
-    <mergeCell ref="M95:N95"/>
-    <mergeCell ref="O95:P95"/>
-    <mergeCell ref="Q95:R95"/>
-    <mergeCell ref="S95:T95"/>
-    <mergeCell ref="U95:V95"/>
-    <mergeCell ref="W86:X86"/>
-    <mergeCell ref="Y86:Z86"/>
-    <mergeCell ref="AA86:AB86"/>
-    <mergeCell ref="AC86:AD86"/>
-    <mergeCell ref="I86:J86"/>
-    <mergeCell ref="K86:L86"/>
-    <mergeCell ref="M86:N86"/>
-    <mergeCell ref="O86:P86"/>
-    <mergeCell ref="Q86:R86"/>
-    <mergeCell ref="S86:T86"/>
-    <mergeCell ref="U86:V86"/>
-    <mergeCell ref="W85:X85"/>
-    <mergeCell ref="Y85:Z85"/>
-    <mergeCell ref="AA85:AB85"/>
-    <mergeCell ref="AC85:AD85"/>
-    <mergeCell ref="I85:J85"/>
-    <mergeCell ref="K85:L85"/>
-    <mergeCell ref="M85:N85"/>
-    <mergeCell ref="O85:P85"/>
-    <mergeCell ref="Q85:R85"/>
-    <mergeCell ref="S85:T85"/>
-    <mergeCell ref="U85:V85"/>
-    <mergeCell ref="W76:X76"/>
-    <mergeCell ref="Y76:Z76"/>
-    <mergeCell ref="AA76:AB76"/>
-    <mergeCell ref="AC76:AD76"/>
-    <mergeCell ref="I76:J76"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="M76:N76"/>
-    <mergeCell ref="O76:P76"/>
-    <mergeCell ref="Q76:R76"/>
-    <mergeCell ref="S76:T76"/>
-    <mergeCell ref="U76:V76"/>
-    <mergeCell ref="W75:X75"/>
-    <mergeCell ref="Y75:Z75"/>
-    <mergeCell ref="AA75:AB75"/>
-    <mergeCell ref="AC75:AD75"/>
-    <mergeCell ref="I75:J75"/>
-    <mergeCell ref="K75:L75"/>
-    <mergeCell ref="M75:N75"/>
-    <mergeCell ref="O75:P75"/>
-    <mergeCell ref="Q75:R75"/>
-    <mergeCell ref="S75:T75"/>
-    <mergeCell ref="U75:V75"/>
-    <mergeCell ref="W66:X66"/>
-    <mergeCell ref="Y66:Z66"/>
-    <mergeCell ref="AA66:AB66"/>
-    <mergeCell ref="AC66:AD66"/>
-    <mergeCell ref="I66:J66"/>
-    <mergeCell ref="K66:L66"/>
-    <mergeCell ref="M66:N66"/>
-    <mergeCell ref="O66:P66"/>
-    <mergeCell ref="Q66:R66"/>
-    <mergeCell ref="S66:T66"/>
-    <mergeCell ref="U66:V66"/>
-    <mergeCell ref="W65:X65"/>
-    <mergeCell ref="Y65:Z65"/>
-    <mergeCell ref="AA65:AB65"/>
-    <mergeCell ref="AC65:AD65"/>
-    <mergeCell ref="I65:J65"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="M65:N65"/>
-    <mergeCell ref="O65:P65"/>
-    <mergeCell ref="Q65:R65"/>
-    <mergeCell ref="S65:T65"/>
-    <mergeCell ref="U65:V65"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -23702,6 +23702,62 @@
     <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="70">
+    <mergeCell ref="U92:V92"/>
+    <mergeCell ref="W92:X92"/>
+    <mergeCell ref="I93:J93"/>
+    <mergeCell ref="K93:N93"/>
+    <mergeCell ref="O93:P93"/>
+    <mergeCell ref="Q93:R93"/>
+    <mergeCell ref="S93:T93"/>
+    <mergeCell ref="U93:V93"/>
+    <mergeCell ref="W93:X93"/>
+    <mergeCell ref="I92:J92"/>
+    <mergeCell ref="K92:N92"/>
+    <mergeCell ref="O92:P92"/>
+    <mergeCell ref="Q92:R92"/>
+    <mergeCell ref="S92:T92"/>
+    <mergeCell ref="U60:V60"/>
+    <mergeCell ref="W60:X60"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="K61:N61"/>
+    <mergeCell ref="O61:P61"/>
+    <mergeCell ref="Q61:R61"/>
+    <mergeCell ref="S61:T61"/>
+    <mergeCell ref="U61:V61"/>
+    <mergeCell ref="W61:X61"/>
+    <mergeCell ref="I60:J60"/>
+    <mergeCell ref="K60:N60"/>
+    <mergeCell ref="O60:P60"/>
+    <mergeCell ref="Q60:R60"/>
+    <mergeCell ref="S60:T60"/>
+    <mergeCell ref="U72:V72"/>
+    <mergeCell ref="W72:X72"/>
+    <mergeCell ref="I73:J73"/>
+    <mergeCell ref="K73:N73"/>
+    <mergeCell ref="O73:P73"/>
+    <mergeCell ref="Q73:R73"/>
+    <mergeCell ref="S73:T73"/>
+    <mergeCell ref="U73:V73"/>
+    <mergeCell ref="W73:X73"/>
+    <mergeCell ref="I72:J72"/>
+    <mergeCell ref="K72:N72"/>
+    <mergeCell ref="O72:P72"/>
+    <mergeCell ref="Q72:R72"/>
+    <mergeCell ref="S72:T72"/>
+    <mergeCell ref="U82:V82"/>
+    <mergeCell ref="W82:X82"/>
+    <mergeCell ref="I83:J83"/>
+    <mergeCell ref="K83:N83"/>
+    <mergeCell ref="O83:P83"/>
+    <mergeCell ref="Q83:R83"/>
+    <mergeCell ref="S83:T83"/>
+    <mergeCell ref="U83:V83"/>
+    <mergeCell ref="W83:X83"/>
+    <mergeCell ref="I82:J82"/>
+    <mergeCell ref="K82:N82"/>
+    <mergeCell ref="O82:P82"/>
+    <mergeCell ref="Q82:R82"/>
+    <mergeCell ref="S82:T82"/>
     <mergeCell ref="U103:V103"/>
     <mergeCell ref="W103:X103"/>
     <mergeCell ref="I102:J102"/>
@@ -23716,62 +23772,6 @@
     <mergeCell ref="O103:P103"/>
     <mergeCell ref="Q103:R103"/>
     <mergeCell ref="S103:T103"/>
-    <mergeCell ref="U82:V82"/>
-    <mergeCell ref="W82:X82"/>
-    <mergeCell ref="I83:J83"/>
-    <mergeCell ref="K83:N83"/>
-    <mergeCell ref="O83:P83"/>
-    <mergeCell ref="Q83:R83"/>
-    <mergeCell ref="S83:T83"/>
-    <mergeCell ref="U83:V83"/>
-    <mergeCell ref="W83:X83"/>
-    <mergeCell ref="I82:J82"/>
-    <mergeCell ref="K82:N82"/>
-    <mergeCell ref="O82:P82"/>
-    <mergeCell ref="Q82:R82"/>
-    <mergeCell ref="S82:T82"/>
-    <mergeCell ref="U72:V72"/>
-    <mergeCell ref="W72:X72"/>
-    <mergeCell ref="I73:J73"/>
-    <mergeCell ref="K73:N73"/>
-    <mergeCell ref="O73:P73"/>
-    <mergeCell ref="Q73:R73"/>
-    <mergeCell ref="S73:T73"/>
-    <mergeCell ref="U73:V73"/>
-    <mergeCell ref="W73:X73"/>
-    <mergeCell ref="I72:J72"/>
-    <mergeCell ref="K72:N72"/>
-    <mergeCell ref="O72:P72"/>
-    <mergeCell ref="Q72:R72"/>
-    <mergeCell ref="S72:T72"/>
-    <mergeCell ref="U60:V60"/>
-    <mergeCell ref="W60:X60"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="K61:N61"/>
-    <mergeCell ref="O61:P61"/>
-    <mergeCell ref="Q61:R61"/>
-    <mergeCell ref="S61:T61"/>
-    <mergeCell ref="U61:V61"/>
-    <mergeCell ref="W61:X61"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="K60:N60"/>
-    <mergeCell ref="O60:P60"/>
-    <mergeCell ref="Q60:R60"/>
-    <mergeCell ref="S60:T60"/>
-    <mergeCell ref="U92:V92"/>
-    <mergeCell ref="W92:X92"/>
-    <mergeCell ref="I93:J93"/>
-    <mergeCell ref="K93:N93"/>
-    <mergeCell ref="O93:P93"/>
-    <mergeCell ref="Q93:R93"/>
-    <mergeCell ref="S93:T93"/>
-    <mergeCell ref="U93:V93"/>
-    <mergeCell ref="W93:X93"/>
-    <mergeCell ref="I92:J92"/>
-    <mergeCell ref="K92:N92"/>
-    <mergeCell ref="O92:P92"/>
-    <mergeCell ref="Q92:R92"/>
-    <mergeCell ref="S92:T92"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.34722222222222221" bottom="0.34722222222222221" header="0.1388888888888889" footer="0.1388888888888889"/>
   <pageSetup scale="89" orientation="landscape" r:id="rId1"/>

</xml_diff>